<commit_message>
muchos cambios, hay un módulo nuevo para el manejo del excel
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -156,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -190,11 +190,20 @@
     <xf borderId="5" fillId="0" fontId="5" numFmtId="11" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="5" numFmtId="11" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="16" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="5" numFmtId="16" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="4" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -214,19 +223,31 @@
     <xf borderId="2" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="2" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="11" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -2470,8 +2491,12 @@
       <c r="E115" s="10">
         <v>435.0</v>
       </c>
-      <c r="F115" s="7"/>
-      <c r="G115" s="7"/>
+      <c r="F115" s="17">
+        <v>65.0</v>
+      </c>
+      <c r="G115" s="17">
+        <v>22.3</v>
+      </c>
       <c r="H115" s="7"/>
       <c r="I115" s="7"/>
       <c r="J115" s="7"/>
@@ -2508,6 +2533,12 @@
       <c r="E116" s="13">
         <v>407.0</v>
       </c>
+      <c r="F116" s="18">
+        <v>66.0</v>
+      </c>
+      <c r="G116" s="18">
+        <v>23.0</v>
+      </c>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="12">
@@ -2525,6 +2556,12 @@
       <c r="E117" s="13">
         <v>392.0</v>
       </c>
+      <c r="F117" s="18">
+        <v>64.0</v>
+      </c>
+      <c r="G117" s="18">
+        <v>23.3</v>
+      </c>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="12">
@@ -2542,6 +2579,12 @@
       <c r="E118" s="13">
         <v>353.0</v>
       </c>
+      <c r="F118" s="18">
+        <v>64.0</v>
+      </c>
+      <c r="G118" s="18">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="12">
@@ -2559,6 +2602,12 @@
       <c r="E119" s="13">
         <v>338.0</v>
       </c>
+      <c r="F119" s="18">
+        <v>64.0</v>
+      </c>
+      <c r="G119" s="18">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="12">
@@ -2576,22 +2625,34 @@
       <c r="E120" s="13">
         <v>329.0</v>
       </c>
+      <c r="F120" s="18">
+        <v>63.0</v>
+      </c>
+      <c r="G120" s="18">
+        <v>24.0</v>
+      </c>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="12">
         <v>46294.0</v>
       </c>
-      <c r="B121" s="17">
+      <c r="B121" s="19">
         <v>35.0</v>
       </c>
-      <c r="C121" s="18">
+      <c r="C121" s="20">
         <v>0.1</v>
       </c>
-      <c r="D121" s="17">
+      <c r="D121" s="19">
         <v>373.0</v>
       </c>
-      <c r="E121" s="17">
+      <c r="E121" s="19">
         <v>320.0</v>
+      </c>
+      <c r="F121" s="18">
+        <v>63.0</v>
+      </c>
+      <c r="G121" s="18">
+        <v>23.6</v>
       </c>
     </row>
     <row r="122" ht="15.75" customHeight="1">
@@ -2610,6 +2671,12 @@
       <c r="E122" s="13">
         <v>306.0</v>
       </c>
+      <c r="F122" s="18">
+        <v>60.0</v>
+      </c>
+      <c r="G122" s="18">
+        <v>24.0</v>
+      </c>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="12">
@@ -2802,16 +2869,16 @@
       <c r="A134" s="12">
         <v>46294.0</v>
       </c>
-      <c r="B134" s="17">
+      <c r="B134" s="19">
         <v>40.0</v>
       </c>
-      <c r="C134" s="18">
+      <c r="C134" s="20">
         <v>0.11</v>
       </c>
-      <c r="D134" s="17">
+      <c r="D134" s="19">
         <v>370.0</v>
       </c>
-      <c r="E134" s="17">
+      <c r="E134" s="19">
         <v>314.0</v>
       </c>
     </row>
@@ -2901,8 +2968,8 @@
       </c>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="A140" s="12">
-        <v>46294.0</v>
+      <c r="A140" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B140" s="13">
         <v>40.0</v>
@@ -2918,8 +2985,8 @@
       </c>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="A141" s="12">
-        <v>46294.0</v>
+      <c r="A141" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B141" s="13">
         <v>40.0</v>
@@ -2935,8 +3002,8 @@
       </c>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="A142" s="12">
-        <v>46294.0</v>
+      <c r="A142" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B142" s="13">
         <v>40.0</v>
@@ -2952,8 +3019,8 @@
       </c>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="A143" s="12">
-        <v>46294.0</v>
+      <c r="A143" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B143" s="13">
         <v>40.0</v>
@@ -2969,8 +3036,8 @@
       </c>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="A144" s="12">
-        <v>46294.0</v>
+      <c r="A144" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B144" s="13">
         <v>40.0</v>
@@ -2986,8 +3053,8 @@
       </c>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="A145" s="12">
-        <v>46294.0</v>
+      <c r="A145" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B145" s="13">
         <v>40.0</v>
@@ -3003,8 +3070,8 @@
       </c>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="A146" s="12">
-        <v>46294.0</v>
+      <c r="A146" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B146" s="13">
         <v>40.0</v>
@@ -3020,8 +3087,8 @@
       </c>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="A147" s="12">
-        <v>46294.0</v>
+      <c r="A147" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B147" s="13">
         <v>40.0</v>
@@ -3037,8 +3104,8 @@
       </c>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="A148" s="12">
-        <v>46294.0</v>
+      <c r="A148" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B148" s="13">
         <v>40.0</v>
@@ -3054,8 +3121,8 @@
       </c>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="A149" s="12">
-        <v>46294.0</v>
+      <c r="A149" s="21">
+        <v>46302.0</v>
       </c>
       <c r="B149" s="13">
         <v>40.0</v>
@@ -3071,138 +3138,138 @@
       </c>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="A150" s="19">
+      <c r="A150" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B150" s="20">
+      <c r="B150" s="23">
         <v>45.0</v>
       </c>
-      <c r="C150" s="21">
+      <c r="C150" s="24">
         <v>0.047</v>
       </c>
-      <c r="D150" s="20">
+      <c r="D150" s="23">
         <v>557.0</v>
       </c>
-      <c r="E150" s="20">
+      <c r="E150" s="23">
         <v>423.0</v>
       </c>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="A151" s="19">
+      <c r="A151" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B151" s="20">
+      <c r="B151" s="23">
         <v>45.0</v>
       </c>
-      <c r="C151" s="21">
+      <c r="C151" s="24">
         <v>0.052</v>
       </c>
-      <c r="D151" s="20">
+      <c r="D151" s="23">
         <v>495.0</v>
       </c>
-      <c r="E151" s="20">
+      <c r="E151" s="23">
         <v>378.0</v>
       </c>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="A152" s="19">
+      <c r="A152" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B152" s="20">
+      <c r="B152" s="23">
         <v>45.0</v>
       </c>
-      <c r="C152" s="21">
+      <c r="C152" s="24">
         <v>0.06</v>
       </c>
-      <c r="D152" s="20">
+      <c r="D152" s="23">
         <v>460.0</v>
       </c>
-      <c r="E152" s="20">
+      <c r="E152" s="23">
         <v>351.0</v>
       </c>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="A153" s="19">
+      <c r="A153" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B153" s="17">
+      <c r="B153" s="19">
         <v>45.0</v>
       </c>
-      <c r="C153" s="18">
+      <c r="C153" s="20">
         <v>0.07</v>
       </c>
-      <c r="D153" s="17">
+      <c r="D153" s="19">
         <v>424.0</v>
       </c>
-      <c r="E153" s="17">
+      <c r="E153" s="19">
         <v>338.0</v>
       </c>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="A154" s="19">
+      <c r="A154" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B154" s="20">
+      <c r="B154" s="23">
         <v>45.0</v>
       </c>
-      <c r="C154" s="21">
+      <c r="C154" s="24">
         <v>0.078</v>
       </c>
-      <c r="D154" s="20">
+      <c r="D154" s="23">
         <v>435.0</v>
       </c>
-      <c r="E154" s="20">
+      <c r="E154" s="23">
         <v>331.0</v>
       </c>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="A155" s="19">
+      <c r="A155" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B155" s="20">
+      <c r="B155" s="23">
         <v>45.0</v>
       </c>
-      <c r="C155" s="21">
+      <c r="C155" s="24">
         <v>0.087</v>
       </c>
-      <c r="D155" s="20">
+      <c r="D155" s="23">
         <v>451.0</v>
       </c>
-      <c r="E155" s="20">
+      <c r="E155" s="23">
         <v>327.0</v>
       </c>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="A156" s="19">
+      <c r="A156" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B156" s="20">
+      <c r="B156" s="23">
         <v>45.0</v>
       </c>
-      <c r="C156" s="21">
+      <c r="C156" s="24">
         <v>0.1</v>
       </c>
-      <c r="D156" s="20">
+      <c r="D156" s="23">
         <v>408.0</v>
       </c>
-      <c r="E156" s="20">
+      <c r="E156" s="23">
         <v>319.0</v>
       </c>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="A157" s="19">
+      <c r="A157" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B157" s="20">
+      <c r="B157" s="23">
         <v>45.0</v>
       </c>
-      <c r="C157" s="21">
+      <c r="C157" s="24">
         <v>0.18</v>
       </c>
-      <c r="D157" s="20">
+      <c r="D157" s="23">
         <v>462.0</v>
       </c>
-      <c r="E157" s="20">
+      <c r="E157" s="23">
         <v>307.0</v>
       </c>
     </row>
@@ -3278,16 +3345,16 @@
       <c r="A162" s="12">
         <v>46294.0</v>
       </c>
-      <c r="B162" s="17">
+      <c r="B162" s="19">
         <v>25.0</v>
       </c>
-      <c r="C162" s="18">
+      <c r="C162" s="20">
         <v>0.17</v>
       </c>
-      <c r="D162" s="17">
+      <c r="D162" s="19">
         <v>363.0</v>
       </c>
-      <c r="E162" s="17">
+      <c r="E162" s="19">
         <v>308.0</v>
       </c>
     </row>
@@ -3394,70 +3461,70 @@
       </c>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="A169" s="19">
+      <c r="A169" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B169" s="20">
+      <c r="B169" s="23">
         <v>15.0</v>
       </c>
-      <c r="C169" s="21">
+      <c r="C169" s="24">
         <v>0.11</v>
       </c>
-      <c r="D169" s="20">
+      <c r="D169" s="23">
         <v>516.0</v>
       </c>
-      <c r="E169" s="20">
+      <c r="E169" s="23">
         <v>421.0</v>
       </c>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="A170" s="19">
+      <c r="A170" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B170" s="20">
+      <c r="B170" s="23">
         <v>15.0</v>
       </c>
-      <c r="C170" s="21">
+      <c r="C170" s="24">
         <v>0.15</v>
       </c>
-      <c r="D170" s="20">
+      <c r="D170" s="23">
         <v>403.0</v>
       </c>
-      <c r="E170" s="20">
+      <c r="E170" s="23">
         <v>348.0</v>
       </c>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="A171" s="19">
+      <c r="A171" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B171" s="20">
+      <c r="B171" s="23">
         <v>15.0</v>
       </c>
-      <c r="C171" s="21">
+      <c r="C171" s="24">
         <v>0.19</v>
       </c>
-      <c r="D171" s="20">
+      <c r="D171" s="23">
         <v>367.0</v>
       </c>
-      <c r="E171" s="20">
+      <c r="E171" s="23">
         <v>321.0</v>
       </c>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="A172" s="19">
+      <c r="A172" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B172" s="20">
+      <c r="B172" s="23">
         <v>15.0</v>
       </c>
-      <c r="C172" s="21">
+      <c r="C172" s="24">
         <v>0.23</v>
       </c>
-      <c r="D172" s="20">
+      <c r="D172" s="23">
         <v>358.0</v>
       </c>
-      <c r="E172" s="20">
+      <c r="E172" s="23">
         <v>311.0</v>
       </c>
     </row>
@@ -3465,118 +3532,118 @@
       <c r="A173" s="12">
         <v>46294.0</v>
       </c>
-      <c r="B173" s="17">
+      <c r="B173" s="19">
         <v>15.0</v>
       </c>
-      <c r="C173" s="18">
+      <c r="C173" s="20">
         <v>0.27</v>
       </c>
-      <c r="D173" s="17">
+      <c r="D173" s="19">
         <v>348.0</v>
       </c>
-      <c r="E173" s="17">
+      <c r="E173" s="19">
         <v>305.0</v>
       </c>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="A174" s="19">
+      <c r="A174" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B174" s="20">
+      <c r="B174" s="23">
         <v>15.0</v>
       </c>
-      <c r="C174" s="21">
+      <c r="C174" s="24">
         <v>0.32</v>
       </c>
-      <c r="D174" s="20">
+      <c r="D174" s="23">
         <v>358.0</v>
       </c>
-      <c r="E174" s="20">
+      <c r="E174" s="23">
         <v>302.0</v>
       </c>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="A175" s="19">
+      <c r="A175" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B175" s="20">
+      <c r="B175" s="23">
         <v>15.0</v>
       </c>
-      <c r="C175" s="21">
+      <c r="C175" s="24">
         <v>0.42</v>
       </c>
-      <c r="D175" s="20">
+      <c r="D175" s="23">
         <v>369.0</v>
       </c>
-      <c r="E175" s="20">
+      <c r="E175" s="23">
         <v>303.0</v>
       </c>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="A176" s="19">
+      <c r="A176" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B176" s="20">
+      <c r="B176" s="23">
         <v>15.0</v>
       </c>
-      <c r="C176" s="21">
+      <c r="C176" s="24">
         <v>0.53</v>
       </c>
-      <c r="D176" s="20">
+      <c r="D176" s="23">
         <v>403.0</v>
       </c>
-      <c r="E176" s="20">
+      <c r="E176" s="23">
         <v>305.0</v>
       </c>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="A177" s="19">
+      <c r="A177" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B177" s="20">
+      <c r="B177" s="23">
         <v>15.0</v>
       </c>
-      <c r="C177" s="21">
+      <c r="C177" s="24">
         <v>0.64</v>
       </c>
-      <c r="D177" s="20">
+      <c r="D177" s="23">
         <v>438.0</v>
       </c>
-      <c r="E177" s="20">
+      <c r="E177" s="23">
         <v>309.0</v>
       </c>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="A178" s="19">
+      <c r="A178" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B178" s="20">
+      <c r="B178" s="23">
         <v>15.0</v>
       </c>
-      <c r="C178" s="21">
+      <c r="C178" s="24">
         <v>0.7</v>
       </c>
-      <c r="D178" s="20">
+      <c r="D178" s="23">
         <v>465.0</v>
       </c>
-      <c r="E178" s="20">
+      <c r="E178" s="23">
         <v>314.0</v>
       </c>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="A179" s="19">
+      <c r="A179" s="22">
         <v>46294.0</v>
       </c>
-      <c r="B179" s="22">
+      <c r="B179" s="25">
         <v>15.0</v>
       </c>
-      <c r="C179" s="23">
+      <c r="C179" s="26">
         <v>0.8</v>
       </c>
-      <c r="D179" s="22">
+      <c r="D179" s="25">
         <v>501.0</v>
       </c>
-      <c r="E179" s="22">
+      <c r="E179" s="25">
         <v>317.0</v>
       </c>
     </row>
@@ -3596,8 +3663,12 @@
       <c r="E180" s="10">
         <v>373.0</v>
       </c>
-      <c r="F180" s="7"/>
-      <c r="G180" s="7"/>
+      <c r="F180" s="17">
+        <v>63.0</v>
+      </c>
+      <c r="G180" s="17">
+        <v>23.6</v>
+      </c>
       <c r="H180" s="7"/>
       <c r="I180" s="7"/>
       <c r="J180" s="7"/>
@@ -3634,6 +3705,12 @@
       <c r="E181" s="13">
         <v>332.0</v>
       </c>
+      <c r="F181" s="18">
+        <v>62.0</v>
+      </c>
+      <c r="G181" s="17">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="3">
@@ -3651,6 +3728,12 @@
       <c r="E182" s="13">
         <v>320.0</v>
       </c>
+      <c r="F182" s="18">
+        <v>61.0</v>
+      </c>
+      <c r="G182" s="18">
+        <v>23.0</v>
+      </c>
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="3">
@@ -3668,6 +3751,12 @@
       <c r="E183" s="13">
         <v>306.0</v>
       </c>
+      <c r="F183" s="18">
+        <v>59.0</v>
+      </c>
+      <c r="G183" s="17">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="3">
@@ -3690,16 +3779,16 @@
       <c r="A185" s="3">
         <v>46295.0</v>
       </c>
-      <c r="B185" s="17">
+      <c r="B185" s="19">
         <v>5.0</v>
       </c>
-      <c r="C185" s="18">
+      <c r="C185" s="20">
         <v>0.72</v>
       </c>
-      <c r="D185" s="17">
+      <c r="D185" s="19">
         <v>339.0</v>
       </c>
-      <c r="E185" s="17">
+      <c r="E185" s="19">
         <v>298.0</v>
       </c>
     </row>
@@ -3772,172 +3861,172 @@
       </c>
     </row>
     <row r="190" ht="15.75" customHeight="1">
-      <c r="A190" s="24">
+      <c r="A190" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B190" s="20">
+      <c r="B190" s="23">
         <v>10.0</v>
       </c>
-      <c r="C190" s="21">
+      <c r="C190" s="24">
         <v>0.18</v>
       </c>
-      <c r="D190" s="20">
+      <c r="D190" s="23">
         <v>476.0</v>
       </c>
-      <c r="E190" s="20">
+      <c r="E190" s="23">
         <v>396.0</v>
       </c>
     </row>
     <row r="191" ht="15.75" customHeight="1">
-      <c r="A191" s="24">
+      <c r="A191" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B191" s="20">
+      <c r="B191" s="23">
         <v>10.0</v>
       </c>
-      <c r="C191" s="21">
+      <c r="C191" s="24">
         <v>0.24</v>
       </c>
-      <c r="D191" s="20">
+      <c r="D191" s="23">
         <v>394.0</v>
       </c>
-      <c r="E191" s="20">
+      <c r="E191" s="23">
         <v>340.0</v>
       </c>
     </row>
     <row r="192" ht="15.75" customHeight="1">
-      <c r="A192" s="24">
+      <c r="A192" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B192" s="20">
+      <c r="B192" s="23">
         <v>10.0</v>
       </c>
-      <c r="C192" s="21">
+      <c r="C192" s="24">
         <v>0.32</v>
       </c>
-      <c r="D192" s="20">
+      <c r="D192" s="23">
         <v>356.0</v>
       </c>
-      <c r="E192" s="20">
+      <c r="E192" s="23">
         <v>310.0</v>
       </c>
     </row>
     <row r="193" ht="15.75" customHeight="1">
-      <c r="A193" s="25">
+      <c r="A193" s="28">
         <v>46295.0</v>
       </c>
-      <c r="B193" s="17">
+      <c r="B193" s="19">
         <v>10.0</v>
       </c>
-      <c r="C193" s="18">
+      <c r="C193" s="20">
         <v>0.42</v>
       </c>
-      <c r="D193" s="17">
+      <c r="D193" s="19">
         <v>354.0</v>
       </c>
-      <c r="E193" s="17">
+      <c r="E193" s="19">
         <v>304.0</v>
       </c>
     </row>
     <row r="194" ht="15.75" customHeight="1">
-      <c r="A194" s="24">
+      <c r="A194" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B194" s="20">
+      <c r="B194" s="23">
         <v>10.0</v>
       </c>
-      <c r="C194" s="21">
+      <c r="C194" s="24">
         <v>0.48</v>
       </c>
-      <c r="D194" s="20">
+      <c r="D194" s="23">
         <v>355.0</v>
       </c>
-      <c r="E194" s="20">
+      <c r="E194" s="23">
         <v>307.0</v>
       </c>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="A195" s="24">
+      <c r="A195" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B195" s="20">
+      <c r="B195" s="23">
         <v>10.0</v>
       </c>
-      <c r="C195" s="21">
+      <c r="C195" s="24">
         <v>0.6</v>
       </c>
-      <c r="D195" s="20">
+      <c r="D195" s="23">
         <v>371.0</v>
       </c>
-      <c r="E195" s="20">
+      <c r="E195" s="23">
         <v>308.0</v>
       </c>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="A196" s="24">
+      <c r="A196" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B196" s="20">
+      <c r="B196" s="23">
         <v>10.0</v>
       </c>
-      <c r="C196" s="21">
+      <c r="C196" s="24">
         <v>0.7</v>
       </c>
-      <c r="D196" s="20">
+      <c r="D196" s="23">
         <v>398.0</v>
       </c>
-      <c r="E196" s="20">
+      <c r="E196" s="23">
         <v>308.0</v>
       </c>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="A197" s="24">
+      <c r="A197" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B197" s="20">
+      <c r="B197" s="23">
         <v>10.0</v>
       </c>
-      <c r="C197" s="21">
+      <c r="C197" s="24">
         <v>0.79</v>
       </c>
-      <c r="D197" s="20">
+      <c r="D197" s="23">
         <v>422.0</v>
       </c>
-      <c r="E197" s="20">
+      <c r="E197" s="23">
         <v>309.0</v>
       </c>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="A198" s="24">
+      <c r="A198" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B198" s="20">
+      <c r="B198" s="23">
         <v>10.0</v>
       </c>
-      <c r="C198" s="21">
+      <c r="C198" s="24">
         <v>0.9</v>
       </c>
-      <c r="D198" s="20">
+      <c r="D198" s="23">
         <v>470.0</v>
       </c>
-      <c r="E198" s="20">
+      <c r="E198" s="23">
         <v>313.0</v>
       </c>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="A199" s="24">
+      <c r="A199" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B199" s="20">
+      <c r="B199" s="23">
         <v>10.0</v>
       </c>
-      <c r="C199" s="21">
+      <c r="C199" s="24">
         <v>0.99</v>
       </c>
-      <c r="D199" s="20">
+      <c r="D199" s="23">
         <v>521.0</v>
       </c>
-      <c r="E199" s="20">
+      <c r="E199" s="23">
         <v>318.0</v>
       </c>
     </row>
@@ -3993,19 +4082,19 @@
       </c>
     </row>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="A203" s="25">
+      <c r="A203" s="28">
         <v>46295.0</v>
       </c>
-      <c r="B203" s="17">
+      <c r="B203" s="19">
         <v>20.0</v>
       </c>
-      <c r="C203" s="18">
+      <c r="C203" s="20">
         <v>0.17</v>
       </c>
-      <c r="D203" s="17">
+      <c r="D203" s="19">
         <v>370.0</v>
       </c>
-      <c r="E203" s="17">
+      <c r="E203" s="19">
         <v>316.0</v>
       </c>
     </row>
@@ -4130,178 +4219,178 @@
       </c>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="A211" s="24">
+      <c r="A211" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B211" s="20">
+      <c r="B211" s="23">
         <v>30.0</v>
       </c>
-      <c r="C211" s="21">
+      <c r="C211" s="24">
         <v>0.069</v>
       </c>
-      <c r="D211" s="20">
+      <c r="D211" s="23">
         <v>437.0</v>
       </c>
-      <c r="E211" s="20">
+      <c r="E211" s="23">
         <v>374.0</v>
       </c>
     </row>
     <row r="212" ht="15.75" customHeight="1">
-      <c r="A212" s="24">
+      <c r="A212" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B212" s="20">
+      <c r="B212" s="23">
         <v>30.0</v>
       </c>
-      <c r="C212" s="21">
+      <c r="C212" s="24">
         <v>0.074</v>
       </c>
-      <c r="D212" s="20">
+      <c r="D212" s="23">
         <v>425.0</v>
       </c>
-      <c r="E212" s="20">
+      <c r="E212" s="23">
         <v>364.0</v>
       </c>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="A213" s="24">
+      <c r="A213" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B213" s="20">
+      <c r="B213" s="23">
         <v>30.0</v>
       </c>
-      <c r="C213" s="21">
+      <c r="C213" s="24">
         <v>0.083</v>
       </c>
-      <c r="D213" s="20">
+      <c r="D213" s="23">
         <v>426.0</v>
       </c>
-      <c r="E213" s="20">
+      <c r="E213" s="23">
         <v>346.0</v>
       </c>
     </row>
     <row r="214" ht="15.75" customHeight="1">
-      <c r="A214" s="24">
+      <c r="A214" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B214" s="20">
+      <c r="B214" s="23">
         <v>30.0</v>
       </c>
-      <c r="C214" s="21">
+      <c r="C214" s="24">
         <v>0.09</v>
       </c>
-      <c r="D214" s="20">
+      <c r="D214" s="23">
         <v>391.0</v>
       </c>
-      <c r="E214" s="20">
+      <c r="E214" s="23">
         <v>339.0</v>
       </c>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="A215" s="25">
+      <c r="A215" s="28">
         <v>46295.0</v>
       </c>
-      <c r="B215" s="17">
+      <c r="B215" s="19">
         <v>30.0</v>
       </c>
-      <c r="C215" s="18">
+      <c r="C215" s="20">
         <v>0.1</v>
       </c>
-      <c r="D215" s="17">
+      <c r="D215" s="19">
         <v>372.0</v>
       </c>
-      <c r="E215" s="17">
+      <c r="E215" s="19">
         <v>326.0</v>
       </c>
     </row>
     <row r="216" ht="15.75" customHeight="1">
-      <c r="A216" s="24">
+      <c r="A216" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B216" s="20">
+      <c r="B216" s="23">
         <v>30.0</v>
       </c>
-      <c r="C216" s="21">
+      <c r="C216" s="24">
         <v>0.14</v>
       </c>
-      <c r="D216" s="20">
+      <c r="D216" s="23">
         <v>372.0</v>
       </c>
-      <c r="E216" s="20">
+      <c r="E216" s="23">
         <v>315.0</v>
       </c>
     </row>
     <row r="217" ht="15.75" customHeight="1">
-      <c r="A217" s="24">
+      <c r="A217" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B217" s="20">
+      <c r="B217" s="23">
         <v>30.0</v>
       </c>
-      <c r="C217" s="21">
+      <c r="C217" s="24">
         <v>0.22</v>
       </c>
-      <c r="D217" s="20">
+      <c r="D217" s="23">
         <v>380.0</v>
       </c>
-      <c r="E217" s="20">
+      <c r="E217" s="23">
         <v>300.0</v>
       </c>
     </row>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="A218" s="24">
+      <c r="A218" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B218" s="20">
+      <c r="B218" s="23">
         <v>30.0</v>
       </c>
-      <c r="C218" s="21">
+      <c r="C218" s="24">
         <v>0.32</v>
       </c>
-      <c r="D218" s="20">
+      <c r="D218" s="23">
         <v>442.0</v>
       </c>
-      <c r="E218" s="20">
+      <c r="E218" s="23">
         <v>309.0</v>
       </c>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="A219" s="24">
+      <c r="A219" s="27">
         <v>46295.0</v>
       </c>
-      <c r="B219" s="22">
+      <c r="B219" s="25">
         <v>30.0</v>
       </c>
-      <c r="C219" s="23">
+      <c r="C219" s="26">
         <v>0.44</v>
       </c>
-      <c r="D219" s="22">
+      <c r="D219" s="25">
         <v>514.0</v>
       </c>
-      <c r="E219" s="22">
+      <c r="E219" s="25">
         <v>330.0</v>
       </c>
     </row>
     <row r="220" ht="15.75" customHeight="1">
-      <c r="A220" s="26">
+      <c r="A220" s="29">
         <v>46301.0</v>
       </c>
-      <c r="B220" s="27">
+      <c r="B220" s="17">
         <v>30.0</v>
       </c>
-      <c r="C220" s="28">
+      <c r="C220" s="30">
         <v>0.056</v>
       </c>
-      <c r="D220" s="27">
+      <c r="D220" s="17">
         <v>563.0</v>
       </c>
-      <c r="E220" s="27">
+      <c r="E220" s="17">
         <v>437.0</v>
       </c>
-      <c r="F220" s="27">
+      <c r="F220" s="17">
         <v>57.0</v>
       </c>
-      <c r="G220" s="27">
+      <c r="G220" s="17">
         <v>23.6</v>
       </c>
       <c r="H220" s="7"/>
@@ -4325,450 +4414,820 @@
       <c r="Z220" s="7"/>
     </row>
     <row r="221" ht="15.75" customHeight="1">
-      <c r="A221" s="29">
+      <c r="A221" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B221" s="30">
+      <c r="B221" s="18">
         <v>30.0</v>
       </c>
-      <c r="C221" s="31">
+      <c r="C221" s="32">
         <v>0.061</v>
       </c>
-      <c r="D221" s="30">
+      <c r="D221" s="18">
         <v>507.0</v>
       </c>
-      <c r="E221" s="30">
+      <c r="E221" s="18">
         <v>403.0</v>
       </c>
-      <c r="F221" s="30">
+      <c r="F221" s="18">
         <v>57.0</v>
       </c>
-      <c r="G221" s="30">
+      <c r="G221" s="18">
         <v>24.3</v>
       </c>
     </row>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="A222" s="29">
+      <c r="A222" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B222" s="30">
+      <c r="B222" s="18">
         <v>30.0</v>
       </c>
-      <c r="C222" s="31">
+      <c r="C222" s="32">
         <v>0.071</v>
       </c>
-      <c r="D222" s="30">
+      <c r="D222" s="18">
         <v>438.0</v>
       </c>
-      <c r="E222" s="30">
+      <c r="E222" s="18">
         <v>367.0</v>
       </c>
+      <c r="F222" s="18">
+        <v>59.0</v>
+      </c>
+      <c r="G222" s="18">
+        <v>23.3</v>
+      </c>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="A223" s="29">
+      <c r="A223" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B223" s="30">
+      <c r="B223" s="18">
         <v>30.0</v>
       </c>
-      <c r="C223" s="31">
+      <c r="C223" s="32">
         <v>0.082</v>
       </c>
-      <c r="D223" s="30">
+      <c r="D223" s="18">
         <v>411.0</v>
       </c>
-      <c r="E223" s="30">
+      <c r="E223" s="18">
         <v>349.0</v>
       </c>
+      <c r="F223" s="18">
+        <v>58.0</v>
+      </c>
+      <c r="G223" s="18">
+        <v>24.0</v>
+      </c>
     </row>
     <row r="224" ht="15.75" customHeight="1">
-      <c r="A224" s="29">
+      <c r="A224" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B224" s="30">
+      <c r="B224" s="18">
         <v>30.0</v>
       </c>
-      <c r="C224" s="31">
+      <c r="C224" s="32">
         <v>0.094</v>
       </c>
-      <c r="D224" s="30">
+      <c r="D224" s="18">
         <v>401.0</v>
       </c>
-      <c r="E224" s="30">
+      <c r="E224" s="18">
         <v>334.0</v>
       </c>
+      <c r="F224" s="18">
+        <v>57.0</v>
+      </c>
+      <c r="G224" s="18">
+        <v>24.3</v>
+      </c>
     </row>
     <row r="225" ht="15.75" customHeight="1">
-      <c r="A225" s="29">
+      <c r="A225" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B225" s="30">
+      <c r="B225" s="18">
         <v>30.0</v>
       </c>
-      <c r="C225" s="31">
+      <c r="C225" s="32">
         <v>0.1</v>
       </c>
-      <c r="D225" s="30">
+      <c r="D225" s="18">
         <v>385.0</v>
       </c>
-      <c r="E225" s="30">
+      <c r="E225" s="18">
         <v>327.0</v>
       </c>
     </row>
     <row r="226" ht="15.75" customHeight="1">
-      <c r="A226" s="29">
+      <c r="A226" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B226" s="30">
+      <c r="B226" s="18">
         <v>30.0</v>
       </c>
-      <c r="C226" s="31">
+      <c r="C226" s="32">
         <v>0.15</v>
       </c>
-      <c r="D226" s="30">
+      <c r="D226" s="18">
         <v>368.0</v>
       </c>
-      <c r="E226" s="30">
+      <c r="E226" s="18">
         <v>310.0</v>
       </c>
     </row>
     <row r="227" ht="15.75" customHeight="1">
-      <c r="A227" s="29">
+      <c r="A227" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B227" s="30">
+      <c r="B227" s="18">
         <v>30.0</v>
       </c>
-      <c r="C227" s="31">
+      <c r="C227" s="32">
         <v>0.2</v>
       </c>
-      <c r="D227" s="30">
+      <c r="D227" s="18">
         <v>383.0</v>
       </c>
-      <c r="E227" s="30">
+      <c r="E227" s="18">
         <v>306.0</v>
       </c>
     </row>
     <row r="228" ht="15.75" customHeight="1">
-      <c r="A228" s="29">
+      <c r="A228" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B228" s="30">
+      <c r="B228" s="18">
         <v>30.0</v>
       </c>
-      <c r="C228" s="31">
+      <c r="C228" s="32">
         <v>0.26</v>
       </c>
-      <c r="D228" s="30">
+      <c r="D228" s="18">
         <v>403.0</v>
       </c>
-      <c r="E228" s="30">
+      <c r="E228" s="18">
         <v>304.0</v>
       </c>
     </row>
     <row r="229" ht="15.75" customHeight="1">
-      <c r="A229" s="29">
+      <c r="A229" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B229" s="30">
+      <c r="B229" s="18">
         <v>30.0</v>
       </c>
-      <c r="C229" s="31">
+      <c r="C229" s="32">
         <v>0.35</v>
       </c>
-      <c r="D229" s="30">
+      <c r="D229" s="18">
         <v>446.0</v>
       </c>
-      <c r="E229" s="30">
+      <c r="E229" s="18">
         <v>310.0</v>
       </c>
     </row>
     <row r="230" ht="15.75" customHeight="1">
-      <c r="A230" s="29">
+      <c r="A230" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B230" s="30">
+      <c r="B230" s="18">
         <v>30.0</v>
       </c>
-      <c r="C230" s="31">
+      <c r="C230" s="32">
         <v>0.44</v>
       </c>
-      <c r="D230" s="30">
+      <c r="D230" s="18">
         <v>494.0</v>
       </c>
-      <c r="E230" s="30">
+      <c r="E230" s="18">
         <v>320.0</v>
       </c>
     </row>
     <row r="231" ht="15.75" customHeight="1">
-      <c r="A231" s="29">
+      <c r="A231" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B231" s="30">
+      <c r="B231" s="18">
         <v>30.0</v>
       </c>
-      <c r="C231" s="31">
+      <c r="C231" s="32">
         <v>0.54</v>
       </c>
-      <c r="D231" s="30">
+      <c r="D231" s="18">
         <v>555.0</v>
       </c>
-      <c r="E231" s="30">
+      <c r="E231" s="18">
         <v>325.0</v>
       </c>
     </row>
     <row r="232" ht="15.75" customHeight="1">
-      <c r="A232" s="29">
+      <c r="A232" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B232" s="30">
+      <c r="B232" s="34">
         <v>35.0</v>
       </c>
-      <c r="C232" s="31">
+      <c r="C232" s="35">
         <v>0.052</v>
       </c>
-      <c r="D232" s="30">
+      <c r="D232" s="34">
         <v>550.0</v>
       </c>
-      <c r="E232" s="30">
+      <c r="E232" s="34">
         <v>421.0</v>
       </c>
     </row>
     <row r="233" ht="15.75" customHeight="1">
-      <c r="A233" s="29">
+      <c r="A233" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B233" s="30">
+      <c r="B233" s="34">
         <v>35.0</v>
       </c>
-      <c r="C233" s="31">
+      <c r="C233" s="35">
         <v>0.056</v>
       </c>
-      <c r="D233" s="30">
+      <c r="D233" s="34">
         <v>496.0</v>
       </c>
-      <c r="E233" s="30">
+      <c r="E233" s="34">
         <v>392.0</v>
       </c>
     </row>
     <row r="234" ht="15.75" customHeight="1">
-      <c r="A234" s="29">
+      <c r="A234" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B234" s="30">
+      <c r="B234" s="34">
         <v>35.0</v>
       </c>
-      <c r="C234" s="31">
+      <c r="C234" s="35">
         <v>0.064</v>
       </c>
-      <c r="D234" s="30">
+      <c r="D234" s="34">
         <v>447.0</v>
       </c>
-      <c r="E234" s="30">
+      <c r="E234" s="34">
         <v>368.0</v>
       </c>
     </row>
     <row r="235" ht="15.75" customHeight="1">
-      <c r="A235" s="29">
+      <c r="A235" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B235" s="30">
+      <c r="B235" s="34">
         <v>35.0</v>
       </c>
-      <c r="C235" s="31">
+      <c r="C235" s="35">
         <v>0.075</v>
       </c>
-      <c r="D235" s="30">
+      <c r="D235" s="34">
         <v>411.0</v>
       </c>
-      <c r="E235" s="30">
+      <c r="E235" s="34">
         <v>346.0</v>
       </c>
     </row>
     <row r="236" ht="15.75" customHeight="1">
-      <c r="A236" s="29">
+      <c r="A236" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B236" s="30">
+      <c r="B236" s="34">
         <v>35.0</v>
       </c>
-      <c r="C236" s="31">
+      <c r="C236" s="35">
         <v>0.083</v>
       </c>
-      <c r="D236" s="30">
+      <c r="D236" s="34">
         <v>396.0</v>
       </c>
-      <c r="E236" s="30">
+      <c r="E236" s="34">
         <v>337.0</v>
       </c>
     </row>
     <row r="237" ht="15.75" customHeight="1">
-      <c r="A237" s="29">
+      <c r="A237" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B237" s="30">
+      <c r="B237" s="34">
         <v>35.0</v>
       </c>
-      <c r="C237" s="31">
+      <c r="C237" s="35">
         <v>0.092</v>
       </c>
-      <c r="D237" s="30">
+      <c r="D237" s="34">
         <v>401.0</v>
       </c>
-      <c r="E237" s="30">
+      <c r="E237" s="34">
         <v>330.0</v>
       </c>
     </row>
     <row r="238" ht="15.75" customHeight="1">
-      <c r="A238" s="29">
+      <c r="A238" s="36">
         <v>46301.0</v>
       </c>
-      <c r="B238" s="30">
+      <c r="B238" s="37">
         <v>35.0</v>
       </c>
-      <c r="C238" s="31">
+      <c r="C238" s="38">
         <v>0.12</v>
       </c>
-      <c r="D238" s="30">
+      <c r="D238" s="37">
         <v>394.0</v>
       </c>
-      <c r="E238" s="30">
+      <c r="E238" s="37">
         <v>316.0</v>
       </c>
     </row>
     <row r="239" ht="15.75" customHeight="1">
-      <c r="A239" s="29">
+      <c r="A239" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B239" s="30">
+      <c r="B239" s="34">
         <v>35.0</v>
       </c>
-      <c r="C239" s="31">
+      <c r="C239" s="35">
         <v>0.16</v>
       </c>
-      <c r="D239" s="30">
+      <c r="D239" s="34">
         <v>384.0</v>
       </c>
-      <c r="E239" s="30">
+      <c r="E239" s="34">
         <v>309.0</v>
       </c>
     </row>
     <row r="240" ht="15.75" customHeight="1">
-      <c r="A240" s="29">
+      <c r="A240" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B240" s="30">
+      <c r="B240" s="34">
         <v>35.0</v>
       </c>
-      <c r="C240" s="31">
+      <c r="C240" s="35">
         <v>0.21</v>
       </c>
-      <c r="D240" s="30">
+      <c r="D240" s="34">
         <v>401.0</v>
       </c>
-      <c r="E240" s="30">
+      <c r="E240" s="34">
         <v>306.0</v>
       </c>
     </row>
     <row r="241" ht="15.75" customHeight="1">
-      <c r="A241" s="29">
+      <c r="A241" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B241" s="30">
+      <c r="B241" s="34">
         <v>35.0</v>
       </c>
-      <c r="C241" s="31">
+      <c r="C241" s="35">
         <v>0.28</v>
       </c>
-      <c r="D241" s="30">
+      <c r="D241" s="34">
         <v>444.0</v>
       </c>
-      <c r="E241" s="30">
+      <c r="E241" s="34">
         <v>308.0</v>
       </c>
     </row>
     <row r="242" ht="15.75" customHeight="1">
-      <c r="A242" s="29">
+      <c r="A242" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B242" s="30">
+      <c r="B242" s="34">
         <v>35.0</v>
       </c>
+      <c r="C242" s="35">
+        <v>0.39</v>
+      </c>
+      <c r="D242" s="34">
+        <v>518.0</v>
+      </c>
+      <c r="E242" s="34">
+        <v>321.0</v>
+      </c>
     </row>
     <row r="243" ht="15.75" customHeight="1">
-      <c r="A243" s="29">
+      <c r="A243" s="33">
         <v>46301.0</v>
       </c>
-      <c r="B243" s="30">
+      <c r="B243" s="34">
         <v>35.0</v>
       </c>
+      <c r="C243" s="35">
+        <v>0.43</v>
+      </c>
+      <c r="D243" s="34">
+        <v>541.0</v>
+      </c>
+      <c r="E243" s="34">
+        <v>323.0</v>
+      </c>
     </row>
     <row r="244" ht="15.75" customHeight="1">
-      <c r="A244" s="29">
+      <c r="A244" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B244" s="30">
-        <v>35.0</v>
+      <c r="B244" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C244" s="32">
+        <v>0.045</v>
+      </c>
+      <c r="D244" s="18">
+        <v>548.0</v>
+      </c>
+      <c r="E244" s="18">
+        <v>426.0</v>
       </c>
     </row>
     <row r="245" ht="15.75" customHeight="1">
-      <c r="A245" s="29">
+      <c r="A245" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B245" s="30">
-        <v>35.0</v>
+      <c r="B245" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C245" s="32">
+        <v>0.053</v>
+      </c>
+      <c r="D245" s="18">
+        <v>457.0</v>
+      </c>
+      <c r="E245" s="18">
+        <v>381.0</v>
       </c>
     </row>
     <row r="246" ht="15.75" customHeight="1">
-      <c r="A246" s="29">
+      <c r="A246" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B246" s="30">
-        <v>35.0</v>
+      <c r="B246" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C246" s="32">
+        <v>0.062</v>
+      </c>
+      <c r="D246" s="18">
+        <v>427.0</v>
+      </c>
+      <c r="E246" s="18">
+        <v>358.0</v>
       </c>
     </row>
     <row r="247" ht="15.75" customHeight="1">
-      <c r="A247" s="29">
+      <c r="A247" s="31">
         <v>46301.0</v>
       </c>
-      <c r="B247" s="30">
-        <v>35.0</v>
+      <c r="B247" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C247" s="32">
+        <v>0.068</v>
+      </c>
+      <c r="D247" s="18">
+        <v>421.0</v>
+      </c>
+      <c r="E247" s="18">
+        <v>347.0</v>
       </c>
     </row>
     <row r="248" ht="15.75" customHeight="1">
-      <c r="A248" s="29">
+      <c r="A248" s="31">
         <v>46301.0</v>
       </c>
+      <c r="B248" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C248" s="32">
+        <v>0.078</v>
+      </c>
+      <c r="D248" s="18">
+        <v>402.0</v>
+      </c>
+      <c r="E248" s="18">
+        <v>337.0</v>
+      </c>
     </row>
     <row r="249" ht="15.75" customHeight="1">
-      <c r="A249" s="29">
+      <c r="A249" s="31">
         <v>46301.0</v>
       </c>
+      <c r="B249" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C249" s="32">
+        <v>0.086</v>
+      </c>
+      <c r="D249" s="18">
+        <v>417.0</v>
+      </c>
+      <c r="E249" s="18">
+        <v>332.0</v>
+      </c>
     </row>
     <row r="250" ht="15.75" customHeight="1">
-      <c r="A250" s="29">
+      <c r="A250" s="31">
         <v>46301.0</v>
       </c>
-    </row>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
+      <c r="B250" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C250" s="32">
+        <v>0.093</v>
+      </c>
+      <c r="D250" s="18">
+        <v>384.0</v>
+      </c>
+      <c r="E250" s="18">
+        <v>327.0</v>
+      </c>
+    </row>
+    <row r="251" ht="15.75" customHeight="1">
+      <c r="A251" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B251" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C251" s="32">
+        <v>0.11</v>
+      </c>
+      <c r="D251" s="18">
+        <v>384.0</v>
+      </c>
+      <c r="E251" s="18">
+        <v>318.0</v>
+      </c>
+    </row>
+    <row r="252" ht="15.75" customHeight="1">
+      <c r="A252" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B252" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C252" s="32">
+        <v>0.19</v>
+      </c>
+      <c r="D252" s="18">
+        <v>419.0</v>
+      </c>
+      <c r="E252" s="18">
+        <v>310.0</v>
+      </c>
+    </row>
+    <row r="253" ht="15.75" customHeight="1">
+      <c r="A253" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B253" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C253" s="32">
+        <v>0.25</v>
+      </c>
+      <c r="D253" s="18">
+        <v>462.0</v>
+      </c>
+      <c r="E253" s="18">
+        <v>310.0</v>
+      </c>
+    </row>
+    <row r="254" ht="15.75" customHeight="1">
+      <c r="A254" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B254" s="18">
+        <v>40.0</v>
+      </c>
+      <c r="C254" s="32">
+        <v>0.36</v>
+      </c>
+      <c r="D254" s="18">
+        <v>534.0</v>
+      </c>
+      <c r="E254" s="18">
+        <v>325.0</v>
+      </c>
+    </row>
+    <row r="255" ht="15.75" customHeight="1">
+      <c r="A255" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B255" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C255" s="32">
+        <v>0.16</v>
+      </c>
+      <c r="D255" s="18">
+        <v>532.0</v>
+      </c>
+      <c r="E255" s="18">
+        <v>433.0</v>
+      </c>
+    </row>
+    <row r="256" ht="15.75" customHeight="1">
+      <c r="A256" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B256" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C256" s="32">
+        <v>0.23</v>
+      </c>
+      <c r="D256" s="18">
+        <v>399.0</v>
+      </c>
+      <c r="E256" s="18">
+        <v>345.0</v>
+      </c>
+    </row>
+    <row r="257" ht="15.75" customHeight="1">
+      <c r="A257" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B257" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C257" s="32">
+        <v>0.28</v>
+      </c>
+      <c r="D257" s="18">
+        <v>372.0</v>
+      </c>
+      <c r="E257" s="18">
+        <v>324.0</v>
+      </c>
+    </row>
+    <row r="258" ht="15.75" customHeight="1">
+      <c r="A258" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B258" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C258" s="32">
+        <v>0.32</v>
+      </c>
+      <c r="D258" s="18">
+        <v>353.0</v>
+      </c>
+      <c r="E258" s="18">
+        <v>311.0</v>
+      </c>
+    </row>
+    <row r="259" ht="15.75" customHeight="1">
+      <c r="A259" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B259" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C259" s="32">
+        <v>0.35</v>
+      </c>
+      <c r="D259" s="18">
+        <v>350.0</v>
+      </c>
+      <c r="E259" s="18">
+        <v>310.0</v>
+      </c>
+    </row>
+    <row r="260" ht="15.75" customHeight="1">
+      <c r="A260" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B260" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C260" s="32">
+        <v>0.42</v>
+      </c>
+      <c r="D260" s="18">
+        <v>351.0</v>
+      </c>
+      <c r="E260" s="18">
+        <v>308.0</v>
+      </c>
+    </row>
+    <row r="261" ht="15.75" customHeight="1">
+      <c r="A261" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B261" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C261" s="32">
+        <v>0.47</v>
+      </c>
+      <c r="D261" s="18">
+        <v>363.0</v>
+      </c>
+      <c r="E261" s="18">
+        <v>308.0</v>
+      </c>
+    </row>
+    <row r="262" ht="15.75" customHeight="1">
+      <c r="A262" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B262" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C262" s="32">
+        <v>0.56</v>
+      </c>
+      <c r="D262" s="18">
+        <v>369.0</v>
+      </c>
+      <c r="E262" s="18">
+        <v>304.0</v>
+      </c>
+    </row>
+    <row r="263" ht="15.75" customHeight="1">
+      <c r="A263" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B263" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C263" s="32">
+        <v>0.65</v>
+      </c>
+      <c r="D263" s="18">
+        <v>384.0</v>
+      </c>
+      <c r="E263" s="18">
+        <v>307.0</v>
+      </c>
+    </row>
+    <row r="264" ht="15.75" customHeight="1">
+      <c r="A264" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B264" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C264" s="32">
+        <v>0.74</v>
+      </c>
+      <c r="D264" s="18">
+        <v>418.0</v>
+      </c>
+      <c r="E264" s="18">
+        <v>312.0</v>
+      </c>
+    </row>
+    <row r="265" ht="15.75" customHeight="1">
+      <c r="A265" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B265" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C265" s="32">
+        <v>0.83</v>
+      </c>
+      <c r="D265" s="18">
+        <v>442.0</v>
+      </c>
+      <c r="E265" s="18">
+        <v>306.0</v>
+      </c>
+    </row>
+    <row r="266" ht="15.75" customHeight="1">
+      <c r="A266" s="31">
+        <v>46301.0</v>
+      </c>
+      <c r="B266" s="18">
+        <v>10.0</v>
+      </c>
+      <c r="C266" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="D266" s="18">
+        <v>482.0</v>
+      </c>
+      <c r="E266" s="18">
+        <v>320.0</v>
+      </c>
+    </row>
+    <row r="267" ht="15.75" customHeight="1">
+      <c r="A267" s="31"/>
+    </row>
+    <row r="268" ht="15.75" customHeight="1">
+      <c r="A268" s="31"/>
+    </row>
+    <row r="269" ht="15.75" customHeight="1">
+      <c r="A269" s="31"/>
+    </row>
     <row r="270" ht="15.75" customHeight="1"/>
     <row r="271" ht="15.75" customHeight="1"/>
     <row r="272" ht="15.75" customHeight="1"/>

</xml_diff>